<commit_message>
Add SQL/DuckDB sheet and sales ZIP column to the pretty demo workbook.
Keep one ODS: reuse Sales/Marketing ranges, put SQL in cells, and join
sheet sales to sibling zip_income.csv via the same generator.

Co-authored-by: KeithCu <KeithCu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/python_showcase_demo.xlsx
+++ b/tests/fixtures/python_showcase_demo.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Optimization" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineering_Math" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Viz_Gallery" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL_DuckDB" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -89,8 +90,13 @@
       <color rgb="00475569"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="000F172A"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -137,6 +143,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F0FDF4"/>
         <bgColor rgb="00F0FDF4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
+        <bgColor rgb="00F1F5F9"/>
       </patternFill>
     </fill>
   </fills>
@@ -194,7 +206,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -240,6 +252,22 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -665,11 +693,11 @@
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="5">
-        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("f'${sum(r[7] for r in data[1:]):,.2f}'", Sales_Analytics!A4:I39)</f>
+        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("f'${sum(r[7] for r in data[1:]):,.2f}'", Sales_Analytics!A4:J39)</f>
         <v/>
       </c>
       <c r="C6" s="5">
-        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("f'{sum(r[7] * (0.28 if r[3]=='Electronics' else 0.30 if r[3]=='Furniture' else 0.22) for r in data[1:]) / sum(r[7] for r in data[1:]):.1%}'", Sales_Analytics!A4:I39)</f>
+        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("f'{sum(r[7] * (0.28 if r[3]=='Electronics' else 0.30 if r[3]=='Furniture' else 0.22) for r in data[1:]) / sum(r[7] for r in data[1:]):.1%}'", Sales_Analytics!A4:J39)</f>
         <v/>
       </c>
       <c r="E6" s="5">
@@ -922,7 +950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -934,6 +962,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -997,6 +1026,11 @@
           <t>SKU_Code</t>
         </is>
       </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>ZIP</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
@@ -1038,6 +1072,11 @@
           <t>ELEC-9021</t>
         </is>
       </c>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>10001</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="11" t="inlineStr">
@@ -1079,6 +1118,11 @@
           <t>FURN-3310</t>
         </is>
       </c>
+      <c r="J6" s="11" t="inlineStr">
+        <is>
+          <t>75201</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
@@ -1120,6 +1164,11 @@
           <t>SUPP-1044</t>
         </is>
       </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>21201</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="11" t="inlineStr">
@@ -1161,6 +1210,11 @@
           <t>ELEC-9042</t>
         </is>
       </c>
+      <c r="J8" s="11" t="inlineStr">
+        <is>
+          <t>80202</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -1202,6 +1256,11 @@
           <t>FURN-3355</t>
         </is>
       </c>
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>10001</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
@@ -1243,6 +1302,11 @@
           <t>ELEC-8812</t>
         </is>
       </c>
+      <c r="J10" s="11" t="inlineStr">
+        <is>
+          <t>20001</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
@@ -1284,6 +1348,11 @@
           <t>SUPP-1089</t>
         </is>
       </c>
+      <c r="J11" s="10" t="inlineStr">
+        <is>
+          <t>33131</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
@@ -1325,6 +1394,11 @@
           <t>FURN-3390</t>
         </is>
       </c>
+      <c r="J12" s="11" t="inlineStr">
+        <is>
+          <t>80202</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
@@ -1366,6 +1440,11 @@
           <t>ELEC-9055</t>
         </is>
       </c>
+      <c r="J13" s="10" t="inlineStr">
+        <is>
+          <t>10001</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="11" t="inlineStr">
@@ -1407,6 +1486,11 @@
           <t>ELEC-9021</t>
         </is>
       </c>
+      <c r="J14" s="11" t="inlineStr">
+        <is>
+          <t>75201</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
@@ -1448,6 +1532,11 @@
           <t>FURN-3320</t>
         </is>
       </c>
+      <c r="J15" s="10" t="inlineStr">
+        <is>
+          <t>21201</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="11" t="inlineStr">
@@ -1489,6 +1578,11 @@
           <t>SUPP-1044</t>
         </is>
       </c>
+      <c r="J16" s="11" t="inlineStr">
+        <is>
+          <t>80202</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -1530,6 +1624,11 @@
           <t>SUPP-1102</t>
         </is>
       </c>
+      <c r="J17" s="10" t="inlineStr">
+        <is>
+          <t>10001</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
@@ -1571,6 +1670,11 @@
           <t>FURN-3310</t>
         </is>
       </c>
+      <c r="J18" s="11" t="inlineStr">
+        <is>
+          <t>75201</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
@@ -1612,6 +1716,11 @@
           <t>ELEC-8830</t>
         </is>
       </c>
+      <c r="J19" s="10" t="inlineStr">
+        <is>
+          <t>21201</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="11" t="inlineStr">
@@ -1653,6 +1762,11 @@
           <t>ELEC-9099</t>
         </is>
       </c>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>80202</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
@@ -1694,6 +1808,11 @@
           <t>FURN-3388</t>
         </is>
       </c>
+      <c r="J21" s="10" t="inlineStr">
+        <is>
+          <t>10001</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="11" t="inlineStr">
@@ -1735,6 +1854,11 @@
           <t>SUPP-1089</t>
         </is>
       </c>
+      <c r="J22" s="11" t="inlineStr">
+        <is>
+          <t>75201</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
@@ -1776,6 +1900,11 @@
           <t>SUPP-1044</t>
         </is>
       </c>
+      <c r="J23" s="10" t="inlineStr">
+        <is>
+          <t>21201</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="11" t="inlineStr">
@@ -1817,6 +1946,11 @@
           <t>FURN-3390</t>
         </is>
       </c>
+      <c r="J24" s="11" t="inlineStr">
+        <is>
+          <t>80202</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
@@ -1858,6 +1992,11 @@
           <t>ELEC-9021</t>
         </is>
       </c>
+      <c r="J25" s="10" t="inlineStr">
+        <is>
+          <t>10001</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="11" t="inlineStr">
@@ -1899,6 +2038,11 @@
           <t>ELEC-8812</t>
         </is>
       </c>
+      <c r="J26" s="11" t="inlineStr">
+        <is>
+          <t>75201</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="10" t="inlineStr">
@@ -1940,6 +2084,11 @@
           <t>FURN-3355</t>
         </is>
       </c>
+      <c r="J27" s="10" t="inlineStr">
+        <is>
+          <t>21201</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="11" t="inlineStr">
@@ -1981,6 +2130,11 @@
           <t>SUPP-1089</t>
         </is>
       </c>
+      <c r="J28" s="11" t="inlineStr">
+        <is>
+          <t>80202</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
@@ -2022,6 +2176,11 @@
           <t>SUPP-1102</t>
         </is>
       </c>
+      <c r="J29" s="10" t="inlineStr">
+        <is>
+          <t>10001</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="11" t="inlineStr">
@@ -2063,6 +2222,11 @@
           <t>FURN-3320</t>
         </is>
       </c>
+      <c r="J30" s="11" t="inlineStr">
+        <is>
+          <t>75201</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="10" t="inlineStr">
@@ -2104,6 +2268,11 @@
           <t>ELEC-9099</t>
         </is>
       </c>
+      <c r="J31" s="10" t="inlineStr">
+        <is>
+          <t>21201</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="11" t="inlineStr">
@@ -2145,6 +2314,11 @@
           <t>ELEC-8830</t>
         </is>
       </c>
+      <c r="J32" s="11" t="inlineStr">
+        <is>
+          <t>80202</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="10" t="inlineStr">
@@ -2186,6 +2360,11 @@
           <t>ELEC-9042</t>
         </is>
       </c>
+      <c r="J33" s="10" t="inlineStr">
+        <is>
+          <t>10001</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="11" t="inlineStr">
@@ -2227,6 +2406,11 @@
           <t>SUPP-1044</t>
         </is>
       </c>
+      <c r="J34" s="11" t="inlineStr">
+        <is>
+          <t>75201</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="10" t="inlineStr">
@@ -2268,6 +2452,11 @@
           <t>SUPP-1089</t>
         </is>
       </c>
+      <c r="J35" s="10" t="inlineStr">
+        <is>
+          <t>21201</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="11" t="inlineStr">
@@ -2309,6 +2498,11 @@
           <t>FURN-3388</t>
         </is>
       </c>
+      <c r="J36" s="11" t="inlineStr">
+        <is>
+          <t>80202</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="10" t="inlineStr">
@@ -2350,6 +2544,11 @@
           <t>FURN-3310</t>
         </is>
       </c>
+      <c r="J37" s="10" t="inlineStr">
+        <is>
+          <t>10001</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="11" t="inlineStr">
@@ -2391,6 +2590,11 @@
           <t>ELEC-9055</t>
         </is>
       </c>
+      <c r="J38" s="11" t="inlineStr">
+        <is>
+          <t>75201</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="10" t="inlineStr">
@@ -2430,6 +2634,11 @@
       <c r="I39" s="10" t="inlineStr">
         <is>
           <t>ELEC-8812</t>
+        </is>
+      </c>
+      <c r="J39" s="10" t="inlineStr">
+        <is>
+          <t>21201</t>
         </is>
       </c>
     </row>
@@ -2448,8 +2657,8 @@
           <t>1. Total Enterprise Sales — Filters and sums all Enterprise tier sales orders</t>
         </is>
       </c>
-      <c r="F43" s="13">
-        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("sum(r[7] for r in data[1:] if r[4]=='Enterprise')", A4:I39)</f>
+      <c r="G43" s="13">
+        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("sum(r[7] for r in data[1:] if r[4]=='Enterprise')", A4:J39)</f>
         <v/>
       </c>
     </row>
@@ -2459,8 +2668,8 @@
           <t>2. Top Revenue SKU — Finds the highest single order revenue SKU code</t>
         </is>
       </c>
-      <c r="F44" s="13">
-        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("max(data[1:], key=lambda r: r[7])[8]", A4:I39)</f>
+      <c r="G44" s="13">
+        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("max(data[1:], key=lambda r: r[7])[8]", A4:J39)</f>
         <v/>
       </c>
     </row>
@@ -2470,8 +2679,8 @@
           <t>3. Avg Units per Order — Calculates average units purchased per transaction</t>
         </is>
       </c>
-      <c r="F45" s="13">
-        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("round(np.mean([r[5] for r in data[1:]]), 1)", A4:I39)</f>
+      <c r="G45" s="13">
+        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("round(np.mean([r[5] for r in data[1:]]), 1)", A4:J39)</f>
         <v/>
       </c>
     </row>
@@ -2481,8 +2690,8 @@
           <t>4. High-Value Threshold (mean plus 2 standard deviations) — Revenue cutoff: mean plus two population standard deviations</t>
         </is>
       </c>
-      <c r="F46" s="13">
-        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("rev = [r[7] for r in data[1:]]; round(np.mean(rev) + 2 * np.std(rev), 2)", A4:I39)</f>
+      <c r="G46" s="13">
+        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("rev = [r[7] for r in data[1:]]; round(np.mean(rev) + 2 * np.std(rev), 2)", A4:J39)</f>
         <v/>
       </c>
     </row>
@@ -2492,26 +2701,26 @@
           <t>5. High Value Orders (above threshold) — Flags orders more than 2 standard deviations above the mean</t>
         </is>
       </c>
-      <c r="F47" s="13">
-        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("sum(r[7] &gt; data[1] for r in data[0][1:])", A4:I39, F46)</f>
+      <c r="G47" s="13">
+        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("sum(r[7] &gt; data[1] for r in data[0][1:])", A4:J39, F46)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A43:E43"/>
-    <mergeCell ref="A42:I42"/>
-    <mergeCell ref="F43:I43"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="F44:I44"/>
-    <mergeCell ref="A47:E47"/>
-    <mergeCell ref="A45:E45"/>
-    <mergeCell ref="A46:E46"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="F47:I47"/>
-    <mergeCell ref="A44:E44"/>
-    <mergeCell ref="F45:I45"/>
-    <mergeCell ref="F46:I46"/>
+    <mergeCell ref="G44:J44"/>
+    <mergeCell ref="G46:J46"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A47:F47"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="A45:F45"/>
+    <mergeCell ref="G43:J43"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="G47:J47"/>
+    <mergeCell ref="A42:J42"/>
+    <mergeCell ref="G45:J45"/>
+    <mergeCell ref="A43:F43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4876,11 +5085,11 @@
           <t>Plot Definition:
 Matplotlib Line Plot — Generates and anchors line chart of order revenues
 Live Formula:
-=ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("plt.figure(figsize=(6,3)); plt.plot([r[7] for r in data[1:]], color='#0284C7', lw=2); plt.title('Sales Revenue Trend'); plt.xlabel('Order #'); plt.ylabel('Revenue ($)'); plt.grid(True, alpha=0.3); plt.tight_layout()", Sales_Analytics!A4:I39)</t>
+=ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("plt.figure(figsize=(6,3)); plt.plot([r[7] for r in data[1:]], color='#0284C7', lw=2); plt.title('Sales Revenue Trend'); plt.xlabel('Order #'); plt.ylabel('Revenue ($)'); plt.grid(True, alpha=0.3); plt.tight_layout()", Sales_Analytics!A4:J39)</t>
         </is>
       </c>
       <c r="D7" s="15">
-        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("plt.figure(figsize=(6,3)); plt.plot([r[7] for r in data[1:]], color='#0284C7', lw=2); plt.title('Sales Revenue Trend'); plt.xlabel('Order #'); plt.ylabel('Revenue ($)'); plt.grid(True, alpha=0.3); plt.tight_layout()", Sales_Analytics!A4:I39)</f>
+        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("plt.figure(figsize=(6,3)); plt.plot([r[7] for r in data[1:]], color='#0284C7', lw=2); plt.title('Sales Revenue Trend'); plt.xlabel('Order #'); plt.ylabel('Revenue ($)'); plt.grid(True, alpha=0.3); plt.tight_layout()", Sales_Analytics!A4:J39)</f>
         <v/>
       </c>
     </row>
@@ -5010,4 +5219,244 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>🦆 SQL / DuckDB — Sheet ranges and sibling files</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Read-only DuckDB SQL over Sales_Analytics / Statistics_ML ranges, plus a join to sibling zip_income.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Sibling zip_income.csv is U.S. Census ACS 2024 5-year table B19013 (median household income; S1903 subject-table equivalent) by ZIP Code Tabulation Area (ZCTA) — reference data you would not keep in the company workbook. Join sales ZIP to that file via query_folder_sql (chat or Run Python Script). Regenerate: python scripts/generate_pretty_demo_spreadsheet.py --format all</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>1. Sheet-only: sales by Region × Category</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>DuckDB GROUP BY on the Sales_Analytics range (no files).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>SQL (edit this text — this is the query)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>SELECT Region, Category,
+       SUM(Revenue) AS revenue,
+       COUNT(*) AS orders
+FROM sales
+GROUP BY Region, Category
+ORDER BY Region, Category</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>RESULTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="36" customHeight="1">
+      <c r="A18" s="20">
+        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("import duckdb; df=pd.DataFrame(data[1:], columns=data[0]); con=duckdb.connect(); con.register('sales', df); result=con.sql("""SELECT Region, Category, SUM(Revenue) AS revenue, COUNT(*) AS orders FROM sales GROUP BY Region, Category ORDER BY Region, Category""").df()", Sales_Analytics!A4:J39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>2. Sheet-only: marketing channel ROAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>Aggregate KPI on the Statistics_ML campaign range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>SQL (edit this text — this is the query)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>SELECT Channel,
+       SUM(Ad_Spend) AS ad_spend,
+       SUM(Revenue) AS revenue,
+       ROUND(SUM(Revenue) / NULLIF(SUM(Ad_Spend), 0), 2) AS roas
+FROM marketing
+GROUP BY Channel
+ORDER BY revenue DESC</t>
+        </is>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>RESULTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="36" customHeight="1">
+      <c r="A31" s="20">
+        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("import duckdb; df=pd.DataFrame(data[1:], columns=data[0]); con=duckdb.connect(); con.register('marketing', df); result=con.sql("""SELECT Channel, SUM(Ad_Spend) AS ad_spend, SUM(Revenue) AS revenue, ROUND(SUM(Revenue) / NULLIF(SUM(Ad_Spend), 0), 2) AS roas FROM marketing GROUP BY Channel ORDER BY revenue DESC""").df()", Statistics_ML!A4:G24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>3. Join: sales ⨝ sibling zip_income.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>Sheet sales ZIP joined to ACS ZCTA median household income. Run via query_folder_sql with tables={sales: Sales_Analytics range} and files={zip_income: zip_income.csv}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="18" t="inlineStr">
+        <is>
+          <t>SQL (edit this text — this is the query)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="19" t="inlineStr">
+        <is>
+          <t>SELECT
+  CASE
+    WHEN z.median_household_income &lt; 75000 THEN 'Under $75k'
+    WHEN z.median_household_income &lt; 120000 THEN '$75k-$120k'
+    ELSE '$120k+'
+  END AS income_band,
+  ROUND(SUM(s.Revenue), 2) AS revenue,
+  ROUND(AVG(z.median_household_income), 0) AS avg_zip_income,
+  COUNT(*) AS orders
+FROM sales s
+JOIN zip_income z
+  ON LPAD(CAST(CAST(ROUND(TRY_CAST(s.ZIP AS DOUBLE)) AS INTEGER) AS VARCHAR), 5, '0')
+   = LPAD(CAST(CAST(ROUND(TRY_CAST(z.zip AS DOUBLE)) AS INTEGER) AS VARCHAR), 5, '0')
+GROUP BY 1
+ORDER BY 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>RESULTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="36" customHeight="1">
+      <c r="A44" s="21" t="inlineStr">
+        <is>
+          <t>Run this SQL with query_folder_sql (preloaded sales + flat_files zip_income). tests/scripting/test_duckdb_sql.py exercises that path against these assets.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="21">
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A24:H28"/>
+    <mergeCell ref="A4:H6"/>
+    <mergeCell ref="A11:H15"/>
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A37:H41"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A43:H43"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A44:H44"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A34:H34"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix SQL_DuckDB RESULTS formulas that closed the PY() string early
_duckdb_register_formula embedded SQL in Python triple-double quotes
inside a Calc formula already delimited by "...". The first " terminated
the argument so SUM(...) / COUNT(*) became bare tokens (Err:508).

Quote SQL with single quotes like the other working demo formulas,
regenerate the showcase fixtures, and add a regression test that the
RESULTS payload stays one well-formed quoted string.

Co-authored-by: KeithCu <KeithCu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/python_showcase_demo.xlsx
+++ b/tests/fixtures/python_showcase_demo.xlsx
@@ -5312,7 +5312,7 @@
     </row>
     <row r="18" ht="36" customHeight="1">
       <c r="A18" s="20">
-        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("import duckdb; df=pd.DataFrame(data[1:], columns=data[0]); con=duckdb.connect(); con.register('sales', df); result=con.sql("""SELECT Region, Category, SUM(Revenue) AS revenue, COUNT(*) AS orders FROM sales GROUP BY Region, Category ORDER BY Region, Category""").df()", Sales_Analytics!A4:J39)</f>
+        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("import duckdb; df=pd.DataFrame(data[1:], columns=data[0]); con=duckdb.connect(); con.register('sales', df); result=con.sql('SELECT Region, Category, SUM(Revenue) AS revenue, COUNT(*) AS orders FROM sales GROUP BY Region, Category ORDER BY Region, Category').df()", Sales_Analytics!A4:J39)</f>
         <v/>
       </c>
     </row>
@@ -5366,7 +5366,7 @@
     </row>
     <row r="31" ht="36" customHeight="1">
       <c r="A31" s="20">
-        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("import duckdb; df=pd.DataFrame(data[1:], columns=data[0]); con=duckdb.connect(); con.register('marketing', df); result=con.sql("""SELECT Channel, SUM(Ad_Spend) AS ad_spend, SUM(Revenue) AS revenue, ROUND(SUM(Revenue) / NULLIF(SUM(Ad_Spend), 0), 2) AS roas FROM marketing GROUP BY Channel ORDER BY revenue DESC""").df()", Statistics_ML!A4:G24)</f>
+        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("import duckdb; df=pd.DataFrame(data[1:], columns=data[0]); con=duckdb.connect(); con.register('marketing', df); result=con.sql('SELECT Channel, SUM(Ad_Spend) AS ad_spend, SUM(Revenue) AS revenue, ROUND(SUM(Revenue) / NULLIF(SUM(Ad_Spend), 0), 2) AS roas FROM marketing GROUP BY Channel ORDER BY revenue DESC').df()", Statistics_ML!A4:G24)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Make SQL_DuckDB RESULTS formulas read SQL from a cell range
Sheet-only RESULTS cells are a short =PY() runner: data[0] is the
sheet range, data[1] is the visible SQL block (joined with newlines).
SQL no longer lives inside the formula string, so Calc cannot hit
Err:508 from nested quotes or comma-to-semicolon rewrites. Scenario 3
stays a query_folder_sql pointer because the sibling CSV is not a
Calc argument.

Co-authored-by: KeithCu <KeithCu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/python_showcase_demo.xlsx
+++ b/tests/fixtures/python_showcase_demo.xlsx
@@ -261,7 +261,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1" indent="1"/>
+      <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
@@ -5227,7 +5227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5258,7 +5258,7 @@
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>
-          <t>Sibling zip_income.csv is U.S. Census ACS 2024 5-year table B19013 (median household income; S1903 subject-table equivalent) by ZIP Code Tabulation Area (ZCTA) — reference data you would not keep in the company workbook. Join sales ZIP to that file via query_folder_sql (chat or Run Python Script). Regenerate: python scripts/generate_pretty_demo_spreadsheet.py --format all</t>
+          <t>Sibling zip_income.csv is U.S. Census ACS 2024 5-year table B19013 (median household income; S1903 subject-table equivalent) by ZIP Code Tabulation Area (ZCTA) — reference data you would not keep in the company workbook. Sheet-only RESULTS: =PY(short code, data_range, sql_range) — data[0] is the sheet range, data[1] is the SQL cells above (joined with newlines). The ZIP join is query_folder_sql (chat or Run Python Script), not a live =PY(), because the CSV is not a Calc argument. Regenerate: python scripts/generate_pretty_demo_spreadsheet.py --format all</t>
         </is>
       </c>
     </row>
@@ -5275,7 +5275,7 @@
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
-          <t>DuckDB GROUP BY on the Sales_Analytics range (no files).</t>
+          <t>DuckDB GROUP BY on the Sales_Analytics range (no files). Edit the SQL cells — RESULTS reads that range via =PY().</t>
         </is>
       </c>
     </row>
@@ -5286,176 +5286,339 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="18" customHeight="1">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>SELECT Region, Category,
-       SUM(Revenue) AS revenue,
-       COUNT(*) AS orders
-FROM sales
-GROUP BY Region, Category
-ORDER BY Region, Category</t>
-        </is>
-      </c>
-    </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+          <t>SELECT Region, Category,</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">       SUM(Revenue) AS revenue,</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">       COUNT(*) AS orders</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>FROM sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>GROUP BY Region, Category</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>ORDER BY Region, Category</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>RESULTS</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="36" customHeight="1">
-      <c r="A18" s="20">
-        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("import duckdb; df=pd.DataFrame(data[1:], columns=data[0]); con=duckdb.connect(); con.register('sales', df); result=con.sql('SELECT Region, Category, SUM(Revenue) AS revenue, COUNT(*) AS orders FROM sales GROUP BY Region, Category ORDER BY Region, Category').df()", Sales_Analytics!A4:J39)</f>
+    <row r="19" ht="36" customHeight="1">
+      <c r="A19" s="20">
+        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("sql=chr(10).join(str(c) for r in data[1] for c in r if c); import duckdb; con=duckdb.connect(); con.register('sales', data[0].to_pandas()); result=con.sql(sql).df()", Sales_Analytics!A4:J39, A11:A16)</f>
         <v/>
       </c>
     </row>
-    <row r="19"/>
     <row r="20"/>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+    <row r="21"/>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>2. Sheet-only: marketing channel ROAS</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="17" t="inlineStr">
-        <is>
-          <t>Aggregate KPI on the Statistics_ML campaign range.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="18" t="inlineStr">
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>Aggregate KPI on the Statistics_ML campaign range. Edit the SQL cells — RESULTS reads that range via =PY().</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
         <is>
           <t>SQL (edit this text — this is the query)</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="19" t="inlineStr">
-        <is>
-          <t>SELECT Channel,
-       SUM(Ad_Spend) AS ad_spend,
-       SUM(Revenue) AS revenue,
-       ROUND(SUM(Revenue) / NULLIF(SUM(Ad_Spend), 0), 2) AS roas
-FROM marketing
-GROUP BY Channel
-ORDER BY revenue DESC</t>
-        </is>
-      </c>
-    </row>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>SELECT Channel,</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">       SUM(Ad_Spend) AS ad_spend,</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">       SUM(Revenue) AS revenue,</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">       ROUND(SUM(Revenue) / NULLIF(SUM(Ad_Spend), 0), 2) AS roas</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="19" t="inlineStr">
+        <is>
+          <t>FROM marketing</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>GROUP BY Channel</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="19" t="inlineStr">
+        <is>
+          <t>ORDER BY revenue DESC</t>
+        </is>
+      </c>
+    </row>
+    <row r="32"/>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>RESULTS</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="36" customHeight="1">
-      <c r="A31" s="20">
-        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("import duckdb; df=pd.DataFrame(data[1:], columns=data[0]); con=duckdb.connect(); con.register('marketing', df); result=con.sql('SELECT Channel, SUM(Ad_Spend) AS ad_spend, SUM(Revenue) AS revenue, ROUND(SUM(Revenue) / NULLIF(SUM(Ad_Spend), 0), 2) AS roas FROM marketing GROUP BY Channel ORDER BY revenue DESC').df()", Statistics_ML!A4:G24)</f>
+    <row r="34" ht="36" customHeight="1">
+      <c r="A34" s="20">
+        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("sql=chr(10).join(str(c) for r in data[1] for c in r if c); import duckdb; con=duckdb.connect(); con.register('marketing', data[0].to_pandas()); result=con.sql(sql).df()", Statistics_ML!A4:G24, A25:A31)</f>
         <v/>
       </c>
     </row>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="3" t="inlineStr">
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>3. Join: sales ⨝ sibling zip_income.csv</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="28" customHeight="1">
-      <c r="A35" s="17" t="inlineStr">
+    <row r="38" ht="28" customHeight="1">
+      <c r="A38" s="17" t="inlineStr">
         <is>
           <t>Sheet sales ZIP joined to ACS ZCTA median household income. Run via query_folder_sql with tables={sales: Sales_Analytics range} and files={zip_income: zip_income.csv}.</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="18" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="18" t="inlineStr">
         <is>
           <t>SQL (edit this text — this is the query)</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="19" t="inlineStr">
-        <is>
-          <t>SELECT
-  CASE
-    WHEN z.median_household_income &lt; 75000 THEN 'Under $75k'
-    WHEN z.median_household_income &lt; 120000 THEN '$75k-$120k'
-    ELSE '$120k+'
-  END AS income_band,
-  ROUND(SUM(s.Revenue), 2) AS revenue,
-  ROUND(AVG(z.median_household_income), 0) AS avg_zip_income,
-  COUNT(*) AS orders
-FROM sales s
-JOIN zip_income z
-  ON LPAD(CAST(CAST(ROUND(TRY_CAST(s.ZIP AS DOUBLE)) AS INTEGER) AS VARCHAR), 5, '0')
-   = LPAD(CAST(CAST(ROUND(TRY_CAST(z.zip AS DOUBLE)) AS INTEGER) AS VARCHAR), 5, '0')
-GROUP BY 1
-ORDER BY 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="19" t="inlineStr">
+        <is>
+          <t>SELECT</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CASE</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    WHEN z.median_household_income &lt; 75000 THEN 'Under $75k'</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    WHEN z.median_household_income &lt; 120000 THEN '$75k-$120k'</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ELSE '$120k+'</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  END AS income_band,</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ROUND(SUM(s.Revenue), 2) AS revenue,</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ROUND(AVG(z.median_household_income), 0) AS avg_zip_income,</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  COUNT(*) AS orders</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="19" t="inlineStr">
+        <is>
+          <t>FROM sales s</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="19" t="inlineStr">
+        <is>
+          <t>JOIN zip_income z</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ON LPAD(CAST(CAST(ROUND(TRY_CAST(s.ZIP AS DOUBLE)) AS INTEGER) AS VARCHAR), 5, '0')</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   = LPAD(CAST(CAST(ROUND(TRY_CAST(z.zip AS DOUBLE)) AS INTEGER) AS VARCHAR), 5, '0')</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="19" t="inlineStr">
+        <is>
+          <t>GROUP BY 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="19" t="inlineStr">
+        <is>
+          <t>ORDER BY 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="55"/>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>RESULTS</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="36" customHeight="1">
-      <c r="A44" s="21" t="inlineStr">
+    <row r="57" ht="36" customHeight="1">
+      <c r="A57" s="21" t="inlineStr">
         <is>
           <t>Run this SQL with query_folder_sql (preloaded sales + flat_files zip_income). tests/scripting/test_duckdb_sql.py exercises that path against these assets.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="46">
     <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A48:H48"/>
     <mergeCell ref="A30:H30"/>
-    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="A39:H39"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A51:H51"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A49:H49"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A24:H28"/>
-    <mergeCell ref="A4:H6"/>
-    <mergeCell ref="A11:H15"/>
+    <mergeCell ref="A45:H45"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A54:H54"/>
+    <mergeCell ref="A41:H41"/>
+    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A46:H46"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A12:H12"/>
     <mergeCell ref="A18:H18"/>
-    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A50:H50"/>
+    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A56:H56"/>
+    <mergeCell ref="A57:H57"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A37:H41"/>
+    <mergeCell ref="A42:H42"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A47:H47"/>
     <mergeCell ref="A23:H23"/>
     <mergeCell ref="A8:H8"/>
     <mergeCell ref="A22:H22"/>
-    <mergeCell ref="A17:H17"/>
-    <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A40:H40"/>
+    <mergeCell ref="A53:H53"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A34:H34"/>
     <mergeCell ref="A43:H43"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A52:H52"/>
     <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A19:H19"/>
     <mergeCell ref="A44:H44"/>
     <mergeCell ref="A31:H31"/>
-    <mergeCell ref="A34:H34"/>
+    <mergeCell ref="A4:H6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leave a 13-row gutter under SQL_DuckDB sheet-only RESULTS
Region×Category spill is header plus 12 data rows. Two empty rows under
A19 put scenario 2's title at A22, which would #SPILL! once auto-spill
works. ODS/XLSX generators now insert SQL_RESULTS_SPILL_GUTTER_ROWS
under live RESULTS; join stays compact. Fixtures regenerated.

Co-authored-by: KeithCu <KeithCu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/python_showcase_demo.xlsx
+++ b/tests/fixtures/python_showcase_demo.xlsx
@@ -5227,7 +5227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5344,228 +5344,250 @@
     </row>
     <row r="20"/>
     <row r="21"/>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>2. Sheet-only: marketing channel ROAS</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="28" customHeight="1">
-      <c r="A23" s="17" t="inlineStr">
+    <row r="34" ht="28" customHeight="1">
+      <c r="A34" s="17" t="inlineStr">
         <is>
           <t>Aggregate KPI on the Statistics_ML campaign range. Edit the SQL cells — RESULTS reads that range via =PY().</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="18" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="18" t="inlineStr">
         <is>
           <t>SQL (edit this text — this is the query)</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="19" t="inlineStr">
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="19" t="inlineStr">
         <is>
           <t>SELECT Channel,</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="19" t="inlineStr">
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">       SUM(Ad_Spend) AS ad_spend,</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="19" t="inlineStr">
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">       SUM(Revenue) AS revenue,</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="19" t="inlineStr">
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">       ROUND(SUM(Revenue) / NULLIF(SUM(Ad_Spend), 0), 2) AS roas</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="19" t="inlineStr">
-        <is>
-          <t>FROM marketing</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="19" t="inlineStr">
-        <is>
-          <t>GROUP BY Channel</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="19" t="inlineStr">
-        <is>
-          <t>ORDER BY revenue DESC</t>
-        </is>
-      </c>
-    </row>
-    <row r="32"/>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>RESULTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="36" customHeight="1">
-      <c r="A34" s="20">
-        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("sql=chr(10).join(str(c) for r in data[1] for c in r if c); import duckdb; con=duckdb.connect(); con.register('marketing', data[0].to_pandas()); result=con.sql(sql).df()", Statistics_ML!A4:G24, A25:A31)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37" ht="22" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>3. Join: sales ⨝ sibling zip_income.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="28" customHeight="1">
-      <c r="A38" s="17" t="inlineStr">
-        <is>
-          <t>Sheet sales ZIP joined to ACS ZCTA median household income. Run via query_folder_sql with tables={sales: Sales_Analytics range} and files={zip_income: zip_income.csv}.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="18" t="inlineStr">
-        <is>
-          <t>SQL (edit this text — this is the query)</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="19" t="inlineStr">
         <is>
-          <t>SELECT</t>
+          <t>FROM marketing</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  CASE</t>
+          <t>GROUP BY Channel</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="19" t="inlineStr">
         <is>
+          <t>ORDER BY revenue DESC</t>
+        </is>
+      </c>
+    </row>
+    <row r="43"/>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>RESULTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="36" customHeight="1">
+      <c r="A45" s="20">
+        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("sql=chr(10).join(str(c) for r in data[1] for c in r if c); import duckdb; con=duckdb.connect(); con.register('marketing', data[0].to_pandas()); result=con.sql(sql).df()", Statistics_ML!A4:G24, A36:A42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>3. Join: sales ⨝ sibling zip_income.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="28" customHeight="1">
+      <c r="A60" s="17" t="inlineStr">
+        <is>
+          <t>Sheet sales ZIP joined to ACS ZCTA median household income. Run via query_folder_sql with tables={sales: Sales_Analytics range} and files={zip_income: zip_income.csv}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="18" t="inlineStr">
+        <is>
+          <t>SQL (edit this text — this is the query)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="19" t="inlineStr">
+        <is>
+          <t>SELECT</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="18" customHeight="1">
+      <c r="A63" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CASE</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="18" customHeight="1">
+      <c r="A64" s="19" t="inlineStr">
+        <is>
           <t xml:space="preserve">    WHEN z.median_household_income &lt; 75000 THEN 'Under $75k'</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="19" t="inlineStr">
+    <row r="65" ht="18" customHeight="1">
+      <c r="A65" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">    WHEN z.median_household_income &lt; 120000 THEN '$75k-$120k'</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="19" t="inlineStr">
+    <row r="66" ht="18" customHeight="1">
+      <c r="A66" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">    ELSE '$120k+'</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="19" t="inlineStr">
+    <row r="67" ht="18" customHeight="1">
+      <c r="A67" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  END AS income_band,</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="19" t="inlineStr">
+    <row r="68" ht="18" customHeight="1">
+      <c r="A68" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  ROUND(SUM(s.Revenue), 2) AS revenue,</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="19" t="inlineStr">
+    <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  ROUND(AVG(z.median_household_income), 0) AS avg_zip_income,</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="19" t="inlineStr">
+    <row r="70" ht="18" customHeight="1">
+      <c r="A70" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  COUNT(*) AS orders</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="19" t="inlineStr">
+    <row r="71" ht="18" customHeight="1">
+      <c r="A71" s="19" t="inlineStr">
         <is>
           <t>FROM sales s</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="19" t="inlineStr">
+    <row r="72" ht="18" customHeight="1">
+      <c r="A72" s="19" t="inlineStr">
         <is>
           <t>JOIN zip_income z</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="19" t="inlineStr">
+    <row r="73" ht="18" customHeight="1">
+      <c r="A73" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  ON LPAD(CAST(CAST(ROUND(TRY_CAST(s.ZIP AS DOUBLE)) AS INTEGER) AS VARCHAR), 5, '0')</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="19" t="inlineStr">
+    <row r="74" ht="18" customHeight="1">
+      <c r="A74" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">   = LPAD(CAST(CAST(ROUND(TRY_CAST(z.zip AS DOUBLE)) AS INTEGER) AS VARCHAR), 5, '0')</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="19" t="inlineStr">
+    <row r="75" ht="18" customHeight="1">
+      <c r="A75" s="19" t="inlineStr">
         <is>
           <t>GROUP BY 1</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="19" t="inlineStr">
+    <row r="76" ht="18" customHeight="1">
+      <c r="A76" s="19" t="inlineStr">
         <is>
           <t>ORDER BY 1</t>
         </is>
       </c>
     </row>
-    <row r="55"/>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+    <row r="77"/>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
         <is>
           <t>RESULTS</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="36" customHeight="1">
-      <c r="A57" s="21" t="inlineStr">
+    <row r="79" ht="36" customHeight="1">
+      <c r="A79" s="21" t="inlineStr">
         <is>
           <t>Run this SQL with query_folder_sql (preloaded sales + flat_files zip_income). tests/scripting/test_duckdb_sql.py exercises that path against these assets.</t>
         </is>
@@ -5574,51 +5596,51 @@
   </sheetData>
   <mergeCells count="46">
     <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A48:H48"/>
-    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A67:H67"/>
     <mergeCell ref="A39:H39"/>
     <mergeCell ref="A15:H15"/>
-    <mergeCell ref="A24:H24"/>
-    <mergeCell ref="A51:H51"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="A73:H73"/>
+    <mergeCell ref="A64:H64"/>
+    <mergeCell ref="A60:H60"/>
+    <mergeCell ref="A36:H36"/>
     <mergeCell ref="A11:H11"/>
-    <mergeCell ref="A49:H49"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A45:H45"/>
-    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A79:H79"/>
+    <mergeCell ref="A61:H61"/>
+    <mergeCell ref="A70:H70"/>
+    <mergeCell ref="A78:H78"/>
+    <mergeCell ref="A69:H69"/>
+    <mergeCell ref="A65:H65"/>
     <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A54:H54"/>
+    <mergeCell ref="A4:H6"/>
     <mergeCell ref="A41:H41"/>
+    <mergeCell ref="A66:H66"/>
     <mergeCell ref="A37:H37"/>
-    <mergeCell ref="A46:H46"/>
-    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A75:H75"/>
+    <mergeCell ref="A74:H74"/>
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="A18:H18"/>
-    <mergeCell ref="A50:H50"/>
-    <mergeCell ref="A26:H26"/>
-    <mergeCell ref="A56:H56"/>
-    <mergeCell ref="A57:H57"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A71:H71"/>
     <mergeCell ref="A42:H42"/>
+    <mergeCell ref="A76:H76"/>
     <mergeCell ref="A33:H33"/>
     <mergeCell ref="A14:H14"/>
-    <mergeCell ref="A47:H47"/>
-    <mergeCell ref="A23:H23"/>
     <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A22:H22"/>
     <mergeCell ref="A40:H40"/>
-    <mergeCell ref="A53:H53"/>
-    <mergeCell ref="A29:H29"/>
-    <mergeCell ref="A34:H34"/>
-    <mergeCell ref="A43:H43"/>
+    <mergeCell ref="A62:H62"/>
+    <mergeCell ref="A35:H35"/>
     <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A52:H52"/>
+    <mergeCell ref="A63:H63"/>
+    <mergeCell ref="A72:H72"/>
     <mergeCell ref="A10:H10"/>
-    <mergeCell ref="A28:H28"/>
     <mergeCell ref="A13:H13"/>
     <mergeCell ref="A19:H19"/>
     <mergeCell ref="A44:H44"/>
-    <mergeCell ref="A31:H31"/>
-    <mergeCell ref="A4:H6"/>
+    <mergeCell ref="A68:H68"/>
+    <mergeCell ref="A34:H34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Unmerge SQL_DuckDB RESULTS cells and reserve a 15x5 spill gutter
Merged A:H / ODS span_cols=8 covered the spill targets so only the
top-left stayed visible. Leave 15 empty rows x 5 cols under each
sheet-only RESULTS (sales worst case is header+12). Keep
result=con.sql(sql).df().

Co-authored-by: KeithCu <KeithCu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/python_showcase_demo.xlsx
+++ b/tests/fixtures/python_showcase_demo.xlsx
@@ -5227,7 +5227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5355,92 +5355,92 @@
     <row r="30"/>
     <row r="31"/>
     <row r="32"/>
-    <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>2. Sheet-only: marketing channel ROAS</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="28" customHeight="1">
-      <c r="A34" s="17" t="inlineStr">
+    <row r="36" ht="28" customHeight="1">
+      <c r="A36" s="17" t="inlineStr">
         <is>
           <t>Aggregate KPI on the Statistics_ML campaign range. Edit the SQL cells — RESULTS reads that range via =PY().</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="18" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="18" t="inlineStr">
         <is>
           <t>SQL (edit this text — this is the query)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="19" t="inlineStr">
-        <is>
-          <t>SELECT Channel,</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       SUM(Ad_Spend) AS ad_spend,</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">       SUM(Revenue) AS revenue,</t>
+          <t>SELECT Channel,</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">       ROUND(SUM(Revenue) / NULLIF(SUM(Ad_Spend), 0), 2) AS roas</t>
+          <t xml:space="preserve">       SUM(Ad_Spend) AS ad_spend,</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="19" t="inlineStr">
         <is>
-          <t>FROM marketing</t>
+          <t xml:space="preserve">       SUM(Revenue) AS revenue,</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="19" t="inlineStr">
         <is>
-          <t>GROUP BY Channel</t>
+          <t xml:space="preserve">       ROUND(SUM(Revenue) / NULLIF(SUM(Ad_Spend), 0), 2) AS roas</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="19" t="inlineStr">
         <is>
+          <t>FROM marketing</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="19" t="inlineStr">
+        <is>
+          <t>GROUP BY Channel</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="19" t="inlineStr">
+        <is>
           <t>ORDER BY revenue DESC</t>
         </is>
       </c>
     </row>
-    <row r="43"/>
-    <row r="44">
-      <c r="A44" s="3" t="inlineStr">
+    <row r="45"/>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>RESULTS</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="36" customHeight="1">
-      <c r="A45" s="20">
-        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("sql=chr(10).join(str(c) for r in data[1] for c in r if c); import duckdb; con=duckdb.connect(); con.register('marketing', data[0].to_pandas()); result=con.sql(sql).df()", Statistics_ML!A4:G24, A36:A42)</f>
+    <row r="47" ht="36" customHeight="1">
+      <c r="A47" s="20">
+        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("sql=chr(10).join(str(c) for r in data[1] for c in r if c); import duckdb; con=duckdb.connect(); con.register('marketing', data[0].to_pandas()); result=con.sql(sql).df()", Statistics_ML!A4:G24, A38:A44)</f>
         <v/>
       </c>
     </row>
-    <row r="46"/>
-    <row r="47"/>
     <row r="48"/>
     <row r="49"/>
     <row r="50"/>
@@ -5452,163 +5452,166 @@
     <row r="56"/>
     <row r="57"/>
     <row r="58"/>
-    <row r="59" ht="22" customHeight="1">
-      <c r="A59" s="3" t="inlineStr">
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="3" t="inlineStr">
         <is>
           <t>3. Join: sales ⨝ sibling zip_income.csv</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="28" customHeight="1">
-      <c r="A60" s="17" t="inlineStr">
+    <row r="64" ht="28" customHeight="1">
+      <c r="A64" s="17" t="inlineStr">
         <is>
           <t>Sheet sales ZIP joined to ACS ZCTA median household income. Run via query_folder_sql with tables={sales: Sales_Analytics range} and files={zip_income: zip_income.csv}.</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="18" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="18" t="inlineStr">
         <is>
           <t>SQL (edit this text — this is the query)</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="18" customHeight="1">
-      <c r="A62" s="19" t="inlineStr">
-        <is>
-          <t>SELECT</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="18" customHeight="1">
-      <c r="A63" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  CASE</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="18" customHeight="1">
-      <c r="A64" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    WHEN z.median_household_income &lt; 75000 THEN 'Under $75k'</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="18" customHeight="1">
-      <c r="A65" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    WHEN z.median_household_income &lt; 120000 THEN '$75k-$120k'</t>
         </is>
       </c>
     </row>
     <row r="66" ht="18" customHeight="1">
       <c r="A66" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ELSE '$120k+'</t>
+          <t>SELECT</t>
         </is>
       </c>
     </row>
     <row r="67" ht="18" customHeight="1">
       <c r="A67" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  END AS income_band,</t>
+          <t xml:space="preserve">  CASE</t>
         </is>
       </c>
     </row>
     <row r="68" ht="18" customHeight="1">
       <c r="A68" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ROUND(SUM(s.Revenue), 2) AS revenue,</t>
+          <t xml:space="preserve">    WHEN z.median_household_income &lt; 75000 THEN 'Under $75k'</t>
         </is>
       </c>
     </row>
     <row r="69" ht="18" customHeight="1">
       <c r="A69" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ROUND(AVG(z.median_household_income), 0) AS avg_zip_income,</t>
+          <t xml:space="preserve">    WHEN z.median_household_income &lt; 120000 THEN '$75k-$120k'</t>
         </is>
       </c>
     </row>
     <row r="70" ht="18" customHeight="1">
       <c r="A70" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  COUNT(*) AS orders</t>
+          <t xml:space="preserve">    ELSE '$120k+'</t>
         </is>
       </c>
     </row>
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="19" t="inlineStr">
         <is>
-          <t>FROM sales s</t>
+          <t xml:space="preserve">  END AS income_band,</t>
         </is>
       </c>
     </row>
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="19" t="inlineStr">
         <is>
-          <t>JOIN zip_income z</t>
+          <t xml:space="preserve">  ROUND(SUM(s.Revenue), 2) AS revenue,</t>
         </is>
       </c>
     </row>
     <row r="73" ht="18" customHeight="1">
       <c r="A73" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ON LPAD(CAST(CAST(ROUND(TRY_CAST(s.ZIP AS DOUBLE)) AS INTEGER) AS VARCHAR), 5, '0')</t>
+          <t xml:space="preserve">  ROUND(AVG(z.median_household_income), 0) AS avg_zip_income,</t>
         </is>
       </c>
     </row>
     <row r="74" ht="18" customHeight="1">
       <c r="A74" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   = LPAD(CAST(CAST(ROUND(TRY_CAST(z.zip AS DOUBLE)) AS INTEGER) AS VARCHAR), 5, '0')</t>
+          <t xml:space="preserve">  COUNT(*) AS orders</t>
         </is>
       </c>
     </row>
     <row r="75" ht="18" customHeight="1">
       <c r="A75" s="19" t="inlineStr">
         <is>
-          <t>GROUP BY 1</t>
+          <t>FROM sales s</t>
         </is>
       </c>
     </row>
     <row r="76" ht="18" customHeight="1">
       <c r="A76" s="19" t="inlineStr">
         <is>
+          <t>JOIN zip_income z</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="18" customHeight="1">
+      <c r="A77" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ON LPAD(CAST(CAST(ROUND(TRY_CAST(s.ZIP AS DOUBLE)) AS INTEGER) AS VARCHAR), 5, '0')</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="18" customHeight="1">
+      <c r="A78" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   = LPAD(CAST(CAST(ROUND(TRY_CAST(z.zip AS DOUBLE)) AS INTEGER) AS VARCHAR), 5, '0')</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="18" customHeight="1">
+      <c r="A79" s="19" t="inlineStr">
+        <is>
+          <t>GROUP BY 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="18" customHeight="1">
+      <c r="A80" s="19" t="inlineStr">
+        <is>
           <t>ORDER BY 1</t>
         </is>
       </c>
     </row>
-    <row r="77"/>
-    <row r="78">
-      <c r="A78" s="3" t="inlineStr">
+    <row r="81"/>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
         <is>
           <t>RESULTS</t>
         </is>
       </c>
     </row>
-    <row r="79" ht="36" customHeight="1">
-      <c r="A79" s="21" t="inlineStr">
+    <row r="83" ht="36" customHeight="1">
+      <c r="A83" s="21" t="inlineStr">
         <is>
           <t>Run this SQL with query_folder_sql (preloaded sales + flat_files zip_income). tests/scripting/test_duckdb_sql.py exercises that path against these assets.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="46">
+  <mergeCells count="44">
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="A67:H67"/>
     <mergeCell ref="A39:H39"/>
+    <mergeCell ref="A77:H77"/>
     <mergeCell ref="A15:H15"/>
-    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="A83:H83"/>
     <mergeCell ref="A73:H73"/>
     <mergeCell ref="A64:H64"/>
-    <mergeCell ref="A60:H60"/>
+    <mergeCell ref="A82:H82"/>
     <mergeCell ref="A36:H36"/>
     <mergeCell ref="A11:H11"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A45:H45"/>
     <mergeCell ref="A79:H79"/>
-    <mergeCell ref="A61:H61"/>
     <mergeCell ref="A70:H70"/>
     <mergeCell ref="A78:H78"/>
     <mergeCell ref="A69:H69"/>
@@ -5617,7 +5620,9 @@
     <mergeCell ref="A4:H6"/>
     <mergeCell ref="A41:H41"/>
     <mergeCell ref="A66:H66"/>
+    <mergeCell ref="A80:H80"/>
     <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A46:H46"/>
     <mergeCell ref="A75:H75"/>
     <mergeCell ref="A74:H74"/>
     <mergeCell ref="A12:H12"/>
@@ -5626,21 +5631,18 @@
     <mergeCell ref="A71:H71"/>
     <mergeCell ref="A42:H42"/>
     <mergeCell ref="A76:H76"/>
-    <mergeCell ref="A33:H33"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A40:H40"/>
-    <mergeCell ref="A62:H62"/>
     <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A43:H43"/>
     <mergeCell ref="A38:H38"/>
     <mergeCell ref="A63:H63"/>
     <mergeCell ref="A72:H72"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A68:H68"/>
     <mergeCell ref="A44:H44"/>
-    <mergeCell ref="A68:H68"/>
-    <mergeCell ref="A34:H34"/>
+    <mergeCell ref="A40:H40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Pretty demo: live ZIP join and {sheet} identity teaching
SQL_DuckDB RESULTS now use named ranges (SalesData / MarketingData)
and session_duckdb() for sheet-only queries. The sales⨝zip_income
join is a live =PY() via run_sql + scoped_dir instead of a pointer.
The sheet teaches {sheet}, {named_range}, and sibling file#Sheet.

Co-authored-by: KeithCu <KeithCu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/python_showcase_demo.xlsx
+++ b/tests/fixtures/python_showcase_demo.xlsx
@@ -16,7 +16,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Viz_Gallery" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL_DuckDB" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="SalesData">Sales_Analytics!A4:J39</definedName>
+    <definedName name="MarketingData">Statistics_ML!A4:G24</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -206,7 +209,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -264,9 +267,6 @@
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
@@ -5227,7 +5227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5250,7 +5250,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Read-only DuckDB SQL over Sales_Analytics / Statistics_ML ranges, plus a join to sibling zip_income.csv</t>
+          <t>Read-only DuckDB SQL over {sheet} / {named_range} identities, plus a live =PY() join to sibling zip_income.csv</t>
         </is>
       </c>
     </row>
@@ -5258,94 +5258,100 @@
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>
-          <t>Sibling zip_income.csv is U.S. Census ACS 2024 5-year table B19013 (median household income; S1903 subject-table equivalent) by ZIP Code Tabulation Area (ZCTA) — reference data you would not keep in the company workbook. Sheet-only RESULTS: =PY(short code, data_range, sql_range) — data[0] is the sheet range, data[1] is the SQL cells above (joined with newlines). The ZIP join is query_folder_sql (chat or Run Python Script), not a live =PY(), because the CSV is not a Calc argument. Regenerate: python scripts/generate_pretty_demo_spreadsheet.py --format all</t>
+          <t>Sibling zip_income.csv is U.S. Census ACS 2024 5-year table B19013 (median household income; S1903 subject-table equivalent) by ZIP Code Tabulation Area (ZCTA) — reference data you would not keep in the company workbook. RESULTS: =PY(short code, data_range, sql_range) — data[0] is the sheet (named range SalesData / MarketingData), data[1] is the SQL cells above (joined with newlines). Sheet-only uses session_duckdb(); the ZIP join is live run_sql(..., files={zip_income: zip_income.csv}, scoped_dir). Prefer catalog identity {sheet: "Sales_Analytics"} (used range), {named_range: "SalesData"}, or sibling file#Sheet (budget.xlsx#Actuals) — not frozen A1. Regenerate: python scripts/generate_pretty_demo_spreadsheet.py --format all</t>
         </is>
       </c>
     </row>
     <row r="5"/>
     <row r="6"/>
     <row r="7"/>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Stable table identity (tool catalog — not frozen A1): {sheet: "Sales_Analytics"} = used range of that sheet; {named_range: "SalesData"} = this workbook's SalesData name; files={zip_income: "zip_income.csv"} = sibling CSV; files={budget: "budget.xlsx#Actuals"} = sibling sheet used range. Live =PY() still passes a Calc name/range so RESULTS dirty when you edit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>1. Sheet-only: sales by Region × Category</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="17" t="inlineStr">
-        <is>
-          <t>DuckDB GROUP BY on the Sales_Analytics range (no files). Edit the SQL cells — RESULTS reads that range via =PY().</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>DuckDB GROUP BY on {sheet: "Sales_Analytics"} / {named_range: "SalesData"} (used-range identity, not frozen A1). Edit the SQL cells — RESULTS reads SalesData via =PY() + session_duckdb().</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>SQL (edit this text — this is the query)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>SELECT Region, Category,</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       SUM(Revenue) AS revenue,</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       COUNT(*) AS orders</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>FROM sales</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="19" t="inlineStr">
         <is>
-          <t>GROUP BY Region, Category</t>
+          <t>SELECT Region, Category,</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="19" t="inlineStr">
         <is>
+          <t xml:space="preserve">       SUM(Revenue) AS revenue,</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">       COUNT(*) AS orders</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>FROM sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>GROUP BY Region, Category</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
           <t>ORDER BY Region, Category</t>
         </is>
       </c>
     </row>
-    <row r="17"/>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>RESULTS</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="36" customHeight="1">
-      <c r="A19" s="20">
-        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("sql=chr(10).join(str(c) for r in data[1] for c in r if c); import duckdb; con=duckdb.connect(); con.register('sales', data[0].to_pandas()); result=con.sql(sql).df()", Sales_Analytics!A4:J39, A11:A16)</f>
+    <row r="23" ht="36" customHeight="1">
+      <c r="A23" s="20">
+        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("sql=chr(10).join(str(c) for r in data[1] for c in r if c); con=session_duckdb(); con.register('sales', data[0].to_pandas()); result=con.sql(sql).df()", SalesData, A15:A20)</f>
         <v/>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
     <row r="24"/>
     <row r="25"/>
     <row r="26"/>
@@ -5357,94 +5363,94 @@
     <row r="32"/>
     <row r="33"/>
     <row r="34"/>
-    <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>2. Sheet-only: marketing channel ROAS</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="28" customHeight="1">
-      <c r="A36" s="17" t="inlineStr">
-        <is>
-          <t>Aggregate KPI on the Statistics_ML campaign range. Edit the SQL cells — RESULTS reads that range via =PY().</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="18" t="inlineStr">
+    <row r="40" ht="28" customHeight="1">
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t>Aggregate KPI on {sheet: "Statistics_ML"} / {named_range: "MarketingData"}. Edit the SQL cells — RESULTS reads MarketingData via =PY() + session_duckdb().</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="18" t="inlineStr">
         <is>
           <t>SQL (edit this text — this is the query)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="19" t="inlineStr">
-        <is>
-          <t>SELECT Channel,</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       SUM(Ad_Spend) AS ad_spend,</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       SUM(Revenue) AS revenue,</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       ROUND(SUM(Revenue) / NULLIF(SUM(Ad_Spend), 0), 2) AS roas</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="19" t="inlineStr">
         <is>
-          <t>FROM marketing</t>
+          <t>SELECT Channel,</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="19" t="inlineStr">
         <is>
-          <t>GROUP BY Channel</t>
+          <t xml:space="preserve">       SUM(Ad_Spend) AS ad_spend,</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="19" t="inlineStr">
         <is>
+          <t xml:space="preserve">       SUM(Revenue) AS revenue,</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">       ROUND(SUM(Revenue) / NULLIF(SUM(Ad_Spend), 0), 2) AS roas</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="19" t="inlineStr">
+        <is>
+          <t>FROM marketing</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="19" t="inlineStr">
+        <is>
+          <t>GROUP BY Channel</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="19" t="inlineStr">
+        <is>
           <t>ORDER BY revenue DESC</t>
         </is>
       </c>
     </row>
-    <row r="45"/>
-    <row r="46">
-      <c r="A46" s="3" t="inlineStr">
+    <row r="49"/>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
         <is>
           <t>RESULTS</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="36" customHeight="1">
-      <c r="A47" s="20">
-        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("sql=chr(10).join(str(c) for r in data[1] for c in r if c); import duckdb; con=duckdb.connect(); con.register('marketing', data[0].to_pandas()); result=con.sql(sql).df()", Statistics_ML!A4:G24, A38:A44)</f>
+    <row r="51" ht="36" customHeight="1">
+      <c r="A51" s="20">
+        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("sql=chr(10).join(str(c) for r in data[1] for c in r if c); con=session_duckdb(); con.register('marketing', data[0].to_pandas()); result=con.sql(sql).df()", MarketingData, A42:A48)</f>
         <v/>
       </c>
     </row>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
     <row r="52"/>
     <row r="53"/>
     <row r="54"/>
@@ -5456,192 +5462,195 @@
     <row r="60"/>
     <row r="61"/>
     <row r="62"/>
-    <row r="63" ht="22" customHeight="1">
-      <c r="A63" s="3" t="inlineStr">
-        <is>
-          <t>3. Join: sales ⨝ sibling zip_income.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="28" customHeight="1">
-      <c r="A64" s="17" t="inlineStr">
-        <is>
-          <t>Sheet sales ZIP joined to ACS ZCTA median household income. Run via query_folder_sql with tables={sales: Sales_Analytics range} and files={zip_income: zip_income.csv}.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="18" t="inlineStr">
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>3. Live join: sales {sheet} ⨝ sibling zip_income.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="28" customHeight="1">
+      <c r="A68" s="17" t="inlineStr">
+        <is>
+          <t>Live =PY() joins {sheet: "Sales_Analytics"} (SalesData) to sibling zip_income.csv via run_sql + scoped_dir. Same catalog as query_folder_sql tables={{sales: {{sheet: "Sales_Analytics"}}}} files={zip_income: zip_income.csv}. Sibling office sheets use file#Sheet (budget.xlsx#Actuals).</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="18" t="inlineStr">
         <is>
           <t>SQL (edit this text — this is the query)</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="18" customHeight="1">
-      <c r="A66" s="19" t="inlineStr">
-        <is>
-          <t>SELECT</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="18" customHeight="1">
-      <c r="A67" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  CASE</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="18" customHeight="1">
-      <c r="A68" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    WHEN z.median_household_income &lt; 75000 THEN 'Under $75k'</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="18" customHeight="1">
-      <c r="A69" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    WHEN z.median_household_income &lt; 120000 THEN '$75k-$120k'</t>
         </is>
       </c>
     </row>
     <row r="70" ht="18" customHeight="1">
       <c r="A70" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ELSE '$120k+'</t>
+          <t>SELECT</t>
         </is>
       </c>
     </row>
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  END AS income_band,</t>
+          <t xml:space="preserve">  CASE</t>
         </is>
       </c>
     </row>
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ROUND(SUM(s.Revenue), 2) AS revenue,</t>
+          <t xml:space="preserve">    WHEN z.median_household_income &lt; 75000 THEN 'Under $75k'</t>
         </is>
       </c>
     </row>
     <row r="73" ht="18" customHeight="1">
       <c r="A73" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ROUND(AVG(z.median_household_income), 0) AS avg_zip_income,</t>
+          <t xml:space="preserve">    WHEN z.median_household_income &lt; 120000 THEN '$75k-$120k'</t>
         </is>
       </c>
     </row>
     <row r="74" ht="18" customHeight="1">
       <c r="A74" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  COUNT(*) AS orders</t>
+          <t xml:space="preserve">    ELSE '$120k+'</t>
         </is>
       </c>
     </row>
     <row r="75" ht="18" customHeight="1">
       <c r="A75" s="19" t="inlineStr">
         <is>
-          <t>FROM sales s</t>
+          <t xml:space="preserve">  END AS income_band,</t>
         </is>
       </c>
     </row>
     <row r="76" ht="18" customHeight="1">
       <c r="A76" s="19" t="inlineStr">
         <is>
-          <t>JOIN zip_income z</t>
+          <t xml:space="preserve">  ROUND(SUM(s.Revenue), 2) AS revenue,</t>
         </is>
       </c>
     </row>
     <row r="77" ht="18" customHeight="1">
       <c r="A77" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ON LPAD(CAST(CAST(ROUND(TRY_CAST(s.ZIP AS DOUBLE)) AS INTEGER) AS VARCHAR), 5, '0')</t>
+          <t xml:space="preserve">  ROUND(AVG(z.median_household_income), 0) AS avg_zip_income,</t>
         </is>
       </c>
     </row>
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   = LPAD(CAST(CAST(ROUND(TRY_CAST(z.zip AS DOUBLE)) AS INTEGER) AS VARCHAR), 5, '0')</t>
+          <t xml:space="preserve">  COUNT(*) AS orders</t>
         </is>
       </c>
     </row>
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="19" t="inlineStr">
         <is>
-          <t>GROUP BY 1</t>
+          <t>FROM sales s</t>
         </is>
       </c>
     </row>
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="19" t="inlineStr">
         <is>
+          <t>JOIN zip_income z</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="18" customHeight="1">
+      <c r="A81" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ON LPAD(CAST(CAST(ROUND(TRY_CAST(s.ZIP AS DOUBLE)) AS INTEGER) AS VARCHAR), 5, '0')</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="18" customHeight="1">
+      <c r="A82" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   = LPAD(CAST(CAST(ROUND(TRY_CAST(z.zip AS DOUBLE)) AS INTEGER) AS VARCHAR), 5, '0')</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="18" customHeight="1">
+      <c r="A83" s="19" t="inlineStr">
+        <is>
+          <t>GROUP BY 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="18" customHeight="1">
+      <c r="A84" s="19" t="inlineStr">
+        <is>
           <t>ORDER BY 1</t>
         </is>
       </c>
     </row>
-    <row r="81"/>
-    <row r="82">
-      <c r="A82" s="3" t="inlineStr">
+    <row r="85"/>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
         <is>
           <t>RESULTS</t>
         </is>
       </c>
     </row>
-    <row r="83" ht="36" customHeight="1">
-      <c r="A83" s="21" t="inlineStr">
-        <is>
-          <t>Run this SQL with query_folder_sql (preloaded sales + flat_files zip_income). tests/scripting/test_duckdb_sql.py exercises that path against these assets.</t>
-        </is>
+    <row r="87" ht="36" customHeight="1">
+      <c r="A87" s="20">
+        <f>ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PY("sql=chr(10).join(str(c) for r in data[1] for c in r if c); result=run_sql(sql,{'sales':data[0]},{'zip_income':'zip_income.csv'},scoped_dir)", SalesData, A70:A84)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="A9:H9"/>
     <mergeCell ref="A67:H67"/>
+    <mergeCell ref="A48:H48"/>
     <mergeCell ref="A39:H39"/>
     <mergeCell ref="A77:H77"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="A83:H83"/>
     <mergeCell ref="A73:H73"/>
-    <mergeCell ref="A64:H64"/>
     <mergeCell ref="A82:H82"/>
-    <mergeCell ref="A36:H36"/>
-    <mergeCell ref="A11:H11"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A45:H45"/>
     <mergeCell ref="A79:H79"/>
     <mergeCell ref="A70:H70"/>
     <mergeCell ref="A78:H78"/>
     <mergeCell ref="A69:H69"/>
-    <mergeCell ref="A65:H65"/>
     <mergeCell ref="A16:H16"/>
     <mergeCell ref="A4:H6"/>
     <mergeCell ref="A41:H41"/>
-    <mergeCell ref="A66:H66"/>
     <mergeCell ref="A80:H80"/>
-    <mergeCell ref="A37:H37"/>
     <mergeCell ref="A46:H46"/>
     <mergeCell ref="A75:H75"/>
+    <mergeCell ref="A84:H84"/>
     <mergeCell ref="A74:H74"/>
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A50:H50"/>
+    <mergeCell ref="A86:H86"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A71:H71"/>
     <mergeCell ref="A42:H42"/>
     <mergeCell ref="A76:H76"/>
     <mergeCell ref="A14:H14"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A47:H47"/>
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A8:H10"/>
+    <mergeCell ref="A20:H20"/>
     <mergeCell ref="A43:H43"/>
-    <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A63:H63"/>
+    <mergeCell ref="A81:H81"/>
     <mergeCell ref="A72:H72"/>
-    <mergeCell ref="A10:H10"/>
     <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A44:H44"/>
     <mergeCell ref="A68:H68"/>
-    <mergeCell ref="A44:H44"/>
     <mergeCell ref="A40:H40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix live-join CalcRange registration and XLSX spill gutter
run_sql must register =PY() CalcRange preloaded tables; bool(range)
is ambiguous and skipped the sales grid. The last XLSX RESULTS is
the ZIP join — add a footer after the 15-row gutter so those rows
exist. Pass doc= in the scoped_dir add-in test.

Co-authored-by: KeithCu <KeithCu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/python_showcase_demo.xlsx
+++ b/tests/fixtures/python_showcase_demo.xlsx
@@ -5227,7 +5227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H87"/>
+  <dimension ref="A1:H103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5606,8 +5606,30 @@
         <v/>
       </c>
     </row>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103" ht="22" customHeight="1">
+      <c r="A103" s="17" t="inlineStr">
+        <is>
+          <t>Edit the SQL cells — live RESULTS recalc through Calc's DAG. Sibling CSV is scoped_dir, not a formula argument.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="44">
+  <mergeCells count="45">
     <mergeCell ref="A67:H67"/>
     <mergeCell ref="A48:H48"/>
     <mergeCell ref="A39:H39"/>
@@ -5618,6 +5640,7 @@
     <mergeCell ref="A82:H82"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A45:H45"/>
+    <mergeCell ref="A103:H103"/>
     <mergeCell ref="A79:H79"/>
     <mergeCell ref="A70:H70"/>
     <mergeCell ref="A78:H78"/>

</xml_diff>

<commit_message>
Fix xlsx =PY named-range packing and scoped_dir inject
Relative XLSX SalesData/MarketingData names shifted when =PY evaluated
them from SQL_DuckDB RESULTS, so data[0] lost headers (Region/Channel).
Write absolute defined names and inject scoped_dir from the cached
calc:file: folder so off-main run_sql joins see the document directory.

Co-authored-by: KeithCu <KeithCu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/python_showcase_demo.xlsx
+++ b/tests/fixtures/python_showcase_demo.xlsx
@@ -17,8 +17,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL_DuckDB" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="SalesData">Sales_Analytics!A4:J39</definedName>
-    <definedName name="MarketingData">Statistics_ML!A4:G24</definedName>
+    <definedName name="SalesData">Sales_Analytics!$A$4:$J$39</definedName>
+    <definedName name="MarketingData">Statistics_ML!$A$4:$G$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>

</xml_diff>